<commit_message>
xanderScript fully implemented. That was alot
</commit_message>
<xml_diff>
--- a/Sizing Code V2/Lookups/engine_lookup.xlsx
+++ b/Sizing Code V2/Lookups/engine_lookup.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\Lookups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing Code V2\Lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AC427C-EBC9-43A6-9692-EE43BA3F20F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E24E00-933E-43B5-90B4-9F6446BD0AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>F404</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>diameter</t>
+  </si>
+  <si>
+    <t>Cost_mil</t>
   </si>
 </sst>
 </file>
@@ -403,17 +406,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
     <col min="2" max="2" width="25.5546875" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="23.44140625" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -424,28 +427,31 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>14</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -455,30 +461,30 @@
       <c r="C2">
         <v>78700</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>26</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>1</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>0.34</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1700</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>45000000</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J2" s="2">
         <f>1035*9.805</f>
         <v>10148.174999999999</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>0.89</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -488,29 +494,29 @@
       <c r="C3">
         <v>191000</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>28</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>1</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>0.56999999999999995</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1700</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>45000000</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>26330</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>1.17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -521,28 +527,31 @@
         <v>92207.185546399996</v>
       </c>
       <c r="D4">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="E4">
         <v>30</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>1</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>0.25</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>1700</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>45000000</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>10045</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>0.89</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -552,30 +561,34 @@
       <c r="C5">
         <v>129600</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
+        <f>6948900/1000000</f>
+        <v>6.9489000000000001</v>
+      </c>
+      <c r="E5">
         <v>32</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>1</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>0.35</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>1700</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>45000000</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <f>1377*9.805</f>
         <v>13501.484999999999</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>0.88</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -585,30 +598,30 @@
       <c r="C6">
         <v>144600</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>30.4</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>0.61</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>1700</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="1">
         <v>45000000</v>
       </c>
-      <c r="I6" s="2">
+      <c r="J6" s="2">
         <f>1740*9.805</f>
         <v>17060.7</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>0.90600000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -618,26 +631,26 @@
       <c r="C7">
         <v>480</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>3</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>1</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>0.1</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>1700</v>
       </c>
-      <c r="H7" s="1">
+      <c r="I7" s="1">
         <v>45000000</v>
       </c>
-      <c r="I7" s="2">
+      <c r="J7" s="2">
         <f>1.65*9.805</f>
         <v>16.178249999999998</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>0.111</v>
       </c>
     </row>

</xml_diff>